<commit_message>
Parameter tuning changes and results for U-Net
</commit_message>
<xml_diff>
--- a/dl/gn/training_results_history.xlsx
+++ b/dl/gn/training_results_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,6 +597,46 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>Baseline for reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-19 03:14:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Weighted BCE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>U-Net (ResNet34 encoder)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1496</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9641999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9418</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.9527</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9101</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>BCE with positive weights to differentiate the small objects in the foreground to the background</t>
         </is>
       </c>
     </row>

</xml_diff>